<commit_message>
Recolor the gptlite-cpp benchmark charts with the site palette
- benchmark.xlsx: the bars of the three charts use the site's blue,
  orange, green and purple, the charts use Helvetica, and the legend
  says PyTorch 2.1.0.
- benchmark_gptlite, benchmark_wide and benchmark_deep are exported from
  the xlsx again, and the post names the new bar colors.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xf6bJex2do3LmU6gkADKZ3
</commit_message>
<xml_diff>
--- a/assets/gptlite-cpp/benchmark.xlsx
+++ b/assets/gptlite-cpp/benchmark.xlsx
@@ -47,7 +47,7 @@
     <t>GPTlite</t>
   </si>
   <si>
-    <t>Pytorch 2.1.0</t>
+    <t>PyTorch 2.1.0</t>
   </si>
   <si>
     <t>PyTorch 1.3.1</t>
@@ -166,7 +166,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -203,7 +203,7 @@
                   <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Helvetica"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
@@ -235,7 +235,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:srgbClr val="6C8EBF"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -265,7 +265,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -350,14 +350,14 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Pytorch 2.1.0</c:v>
+                  <c:v>PyTorch 2.1.0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent2"/>
+              <a:srgbClr val="D79B00"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -387,7 +387,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -479,7 +479,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent3"/>
+              <a:srgbClr val="82B366"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -509,7 +509,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -601,7 +601,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent4"/>
+              <a:srgbClr val="9673A6"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -631,7 +631,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -752,7 +752,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -811,7 +811,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -853,7 +853,7 @@
                   <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Helvetica"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
@@ -922,7 +922,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -959,7 +959,7 @@
                   <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Helvetica"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
@@ -991,7 +991,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:srgbClr val="6C8EBF"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1021,7 +1021,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -1106,14 +1106,14 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Pytorch 2.1.0</c:v>
+                  <c:v>PyTorch 2.1.0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent2"/>
+              <a:srgbClr val="D79B00"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1143,7 +1143,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -1235,7 +1235,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent3"/>
+              <a:srgbClr val="82B366"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1265,7 +1265,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -1357,7 +1357,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent4"/>
+              <a:srgbClr val="9673A6"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1387,7 +1387,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -1508,7 +1508,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -1567,7 +1567,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -1609,7 +1609,7 @@
                   <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Helvetica"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
@@ -1678,7 +1678,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -1710,7 +1710,7 @@
                   <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Helvetica"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
@@ -1742,7 +1742,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:srgbClr val="6C8EBF"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1772,7 +1772,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -1857,14 +1857,14 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Pytorch 2.1.0</c:v>
+                  <c:v>PyTorch 2.1.0</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent2"/>
+              <a:srgbClr val="D79B00"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1894,7 +1894,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -1986,7 +1986,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent3"/>
+              <a:srgbClr val="82B366"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -2016,7 +2016,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -2108,7 +2108,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent4"/>
+              <a:srgbClr val="9673A6"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -2138,7 +2138,7 @@
                         <a:lumOff val="25000"/>
                       </a:schemeClr>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Helvetica"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
@@ -2259,7 +2259,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -2318,7 +2318,7 @@
                     <a:lumOff val="35000"/>
                   </a:schemeClr>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Helvetica"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
@@ -2360,7 +2360,7 @@
                   <a:lumOff val="35000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Helvetica"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>

</xml_diff>

<commit_message>
Name the PyTorch 2.1 versions without the patch number and correct the gain to 19% in gptlite-cpp
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xf6bJex2do3LmU6gkADKZ3
</commit_message>
<xml_diff>
--- a/assets/gptlite-cpp/benchmark.xlsx
+++ b/assets/gptlite-cpp/benchmark.xlsx
@@ -47,13 +47,13 @@
     <t>GPTlite</t>
   </si>
   <si>
-    <t>PyTorch 2.1.0</t>
+    <t>PyTorch 2.1</t>
   </si>
   <si>
     <t>PyTorch 1.3.1</t>
   </si>
   <si>
-    <t>C++ LibTorch 2.1.0</t>
+    <t>C++ LibTorch 2.1</t>
   </si>
   <si>
     <t>inference throughput (samples/sec)</t>
@@ -65,7 +65,7 @@
     <t>memory usage (GB)</t>
   </si>
   <si>
-    <t>TorchScript 2.1.0 (inf. only)</t>
+    <t>TorchScript 2.1 (inf. only)</t>
   </si>
 </sst>
 </file>
@@ -350,7 +350,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>PyTorch 2.1.0</c:v>
+                  <c:v>PyTorch 2.1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -472,7 +472,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>C++ LibTorch 2.1.0</c:v>
+                  <c:v>C++ LibTorch 2.1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -594,7 +594,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TorchScript 2.1.0 (inf. only)</c:v>
+                  <c:v>TorchScript 2.1 (inf. only)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1106,7 +1106,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>PyTorch 2.1.0</c:v>
+                  <c:v>PyTorch 2.1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1228,7 +1228,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>C++ LibTorch 2.1.0</c:v>
+                  <c:v>C++ LibTorch 2.1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1350,7 +1350,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TorchScript 2.1.0 (inf. only)</c:v>
+                  <c:v>TorchScript 2.1 (inf. only)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1857,7 +1857,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>PyTorch 2.1.0</c:v>
+                  <c:v>PyTorch 2.1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1979,7 +1979,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>C++ LibTorch 2.1.0</c:v>
+                  <c:v>C++ LibTorch 2.1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2101,7 +2101,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>TorchScript 2.1.0 (inf. only)</c:v>
+                  <c:v>TorchScript 2.1 (inf. only)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>

</xml_diff>